<commit_message>
removed ineligible users and found replacements
</commit_message>
<xml_diff>
--- a/outputs/replacement_candidates_next_20_with_journals.xlsx
+++ b/outputs/replacement_candidates_next_20_with_journals.xlsx
@@ -571,12 +571,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Jue Herman</t>
+          <t>Sariffudin Fiza</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>856282500</t>
+          <t>25640455475627828</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -599,45 +599,45 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-04-07 19:05:48 GMT+8</t>
+          <t>2026-04-17 15:40:28 GMT+8</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-04-07 19:06:24 GMT+8</t>
+          <t>2026-04-17 16:13:56 GMT+8</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2026-04-07 19:05:15 GMT+8</t>
+          <t>2026-04-17 16:12:47 GMT+8</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2026-04-07 19:04:43 GMT+8</t>
+          <t>2026-04-17 15:39:37 GMT+8</t>
         </is>
       </c>
       <c r="M2" t="n">
-        <v>31157</v>
+        <v>36502</v>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-04-07 19:05:48 GMT+8</t>
+          <t>2026-04-17 15:40:28 GMT+8</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>saya tolong mak saya harini</t>
+          <t>saya sayang family saya</t>
         </is>
       </c>
       <c r="P2" t="n">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="Q2" t="n">
-        <v>15.68</v>
+        <v>-9.43</v>
       </c>
       <c r="R2" t="n">
-        <v>0.6749999999999999</v>
+        <v>0.575</v>
       </c>
       <c r="S2" t="n">
         <v>10</v>
@@ -652,7 +652,7 @@
         <v>0</v>
       </c>
       <c r="W2" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="X2" t="n">
         <v>0</v>
@@ -670,7 +670,7 @@
         <v>0</v>
       </c>
       <c r="AC2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AD2" t="inlineStr">
         <is>
@@ -681,12 +681,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Kamariah Nor</t>
+          <t>Shameel Isfahan</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>45402747</t>
+          <t>25409058178770177</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -709,45 +709,45 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-04-19 13:07:12 GMT+8</t>
+          <t>2026-04-12 09:57:57 GMT+8</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-04-19 13:10:37 GMT+8</t>
+          <t>2026-04-12 10:26:46 GMT+8</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>2026-04-19 13:05:49 GMT+8</t>
+          <t>2026-04-12 09:56:09 GMT+8</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>2026-04-19 13:04:18 GMT+8</t>
+          <t>2026-04-12 09:56:08 GMT+8</t>
         </is>
       </c>
       <c r="M3" t="n">
-        <v>36903</v>
+        <v>33118</v>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-04-19 13:07:12 GMT+8</t>
+          <t>2026-04-12 09:57:57 GMT+8</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Saya suka memberi makanan untuk kucing kucing jalanan</t>
+          <t>Saya suka berlari sambil bersedekah</t>
         </is>
       </c>
       <c r="P3" t="n">
-        <v>53</v>
+        <v>35</v>
       </c>
       <c r="Q3" t="n">
-        <v>6.32</v>
+        <v>5.88</v>
       </c>
       <c r="R3" t="n">
-        <v>1.325</v>
+        <v>0.875</v>
       </c>
       <c r="S3" t="n">
         <v>5</v>
@@ -791,12 +791,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Kam Wai Kwan</t>
+          <t>Shazlin Rosly</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>25230176969988610</t>
+          <t>26809398435345201</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -819,48 +819,48 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-03-27 18:42:15 GMT+8</t>
+          <t>2026-04-12 08:22:19 GMT+8</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-03-27 18:45:05 GMT+8</t>
+          <t>2026-04-12 08:22:53 GMT+8</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>2026-03-27 18:40:36 GMT+8</t>
+          <t>2026-04-12 08:20:50 GMT+8</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>2026-03-27 18:40:35 GMT+8</t>
+          <t>2026-04-12 08:20:49 GMT+8</t>
         </is>
       </c>
       <c r="M4" t="n">
-        <v>23605</v>
+        <v>32871</v>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>2026-03-27 18:45:05 GMT+8</t>
+          <t>2026-04-12 08:22:53 GMT+8</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>Saya mahu menolong datuk &amp; nenek memastikan rumah kemas Dan baru</t>
+          <t>Saya Bantu jiran angkat air</t>
         </is>
       </c>
       <c r="P4" t="n">
-        <v>64</v>
+        <v>27</v>
       </c>
       <c r="Q4" t="n">
-        <v>21.6</v>
+        <v>15.68</v>
       </c>
       <c r="R4" t="n">
-        <v>1.6</v>
+        <v>0.6749999999999999</v>
       </c>
       <c r="S4" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="T4" t="n">
         <v>5</v>
@@ -878,7 +878,7 @@
         <v>0</v>
       </c>
       <c r="Y4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Z4" t="n">
         <v>1</v>
@@ -901,12 +901,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Karan Patel</t>
+          <t>Shera Nazri</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>1826887376</t>
+          <t>187412901</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -929,45 +929,45 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-04-13 21:25:26 GMT+8</t>
+          <t>2026-03-16 05:58:14 GMT+8</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-04-13 21:25:45 GMT+8</t>
+          <t>2026-03-16 05:58:47 GMT+8</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>2026-04-13 21:25:01 GMT+8</t>
+          <t>2026-04-03 13:41:35 GMT+8</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>2026-04-13 21:24:25 GMT+8</t>
+          <t>2026-03-16 05:56:01 GMT+8</t>
         </is>
       </c>
       <c r="M5" t="n">
-        <v>33701</v>
+        <v>14177</v>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>2026-04-13 21:25:26 GMT+8</t>
+          <t>2026-03-16 05:58:47 GMT+8</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Saya bantu rakan membawa buku yang banyak ke kelas.</t>
+          <t>Saya bantu keluarga saya mengecat rumah</t>
         </is>
       </c>
       <c r="P5" t="n">
-        <v>51</v>
+        <v>39</v>
       </c>
       <c r="Q5" t="n">
-        <v>-8.73</v>
+        <v>15.98</v>
       </c>
       <c r="R5" t="n">
-        <v>1.275</v>
+        <v>0.9750000000000001</v>
       </c>
       <c r="S5" t="n">
         <v>10</v>
@@ -982,7 +982,7 @@
         <v>0</v>
       </c>
       <c r="W5" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="X5" t="n">
         <v>0</v>
@@ -1000,7 +1000,7 @@
         <v>0</v>
       </c>
       <c r="AC5" t="n">
-        <v>51</v>
+        <v>1</v>
       </c>
       <c r="AD5" t="inlineStr">
         <is>
@@ -1011,12 +1011,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Kavitha Jaganathan</t>
+          <t>Shira Jalil</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>25953022347654371</t>
+          <t>26304478562497060</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -1039,51 +1039,51 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-03-14 17:14:06 GMT+8</t>
+          <t>2026-03-14 01:22:42 GMT+8</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-03-14 17:15:34 GMT+8</t>
+          <t>2026-03-14 01:24:53 GMT+8</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>2026-03-14 17:11:46 GMT+8</t>
+          <t>2026-03-14 01:24:08 GMT+8</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>2026-03-14 17:11:14 GMT+8</t>
+          <t>2026-03-14 01:21:38 GMT+8</t>
         </is>
       </c>
       <c r="M6" t="n">
-        <v>12816</v>
+        <v>11836</v>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>2026-03-14 17:15:34 GMT+8</t>
+          <t>2026-03-14 01:24:53 GMT+8</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>Saya menyumbang 12 botol Topicana Twister kepada rumah anak yatim berhampiran rumah saya</t>
+          <t>saya suka tolong orang</t>
         </is>
       </c>
       <c r="P6" t="n">
-        <v>88</v>
+        <v>22</v>
       </c>
       <c r="Q6" t="n">
-        <v>-7.8</v>
+        <v>-14.45</v>
       </c>
       <c r="R6" t="n">
-        <v>2.2</v>
+        <v>0.55</v>
       </c>
       <c r="S6" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="T6" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="U6" t="n">
         <v>0</v>
@@ -1092,16 +1092,16 @@
         <v>0</v>
       </c>
       <c r="W6" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="X6" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="Y6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Z6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA6" t="n">
         <v>0</v>
@@ -1110,7 +1110,7 @@
         <v>0</v>
       </c>
       <c r="AC6" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="AD6" t="inlineStr">
         <is>
@@ -1121,12 +1121,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Khawlah Al Azwar</t>
+          <t>Siew</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>26988101557453565</t>
+          <t>765882994</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -1149,48 +1149,48 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-04-11 09:34:12 GMT+8</t>
+          <t>2026-02-20 12:39:13 GMT+8</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-04-11 09:37:06 GMT+8</t>
+          <t>2026-02-20 12:41:25 GMT+8</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>2026-04-11 09:36:16 GMT+8</t>
+          <t>2026-02-20 12:34:32 GMT+8</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>2026-04-11 09:33:10 GMT+8</t>
+          <t>2026-02-20 12:33:49 GMT+8</t>
         </is>
       </c>
       <c r="M7" t="n">
-        <v>32535</v>
+        <v>220</v>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>2026-04-11 09:34:12 GMT+8</t>
+          <t>2026-02-20 12:39:13 GMT+8</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>Sy suka menyeryai run harini...</t>
+          <t>Saya memperkenalkan minuman tropicana Twister kepada kawan sekerja saya. Selain itu, Tropicana Twister merupakan minuman utama tajaan saya kepada jamuan di anak sekolah saya.</t>
         </is>
       </c>
       <c r="P7" t="n">
-        <v>31</v>
+        <v>174</v>
       </c>
       <c r="Q7" t="n">
-        <v>0.78</v>
+        <v>19.35</v>
       </c>
       <c r="R7" t="n">
-        <v>0.775</v>
+        <v>4.35</v>
       </c>
       <c r="S7" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="T7" t="n">
         <v>0</v>
@@ -1208,7 +1208,7 @@
         <v>0</v>
       </c>
       <c r="Y7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="Z7" t="n">
         <v>0</v>
@@ -1231,12 +1231,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Kirtanah Ravintharan</t>
+          <t>Siti Nurhani</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>26327752256875020</t>
+          <t>27099866149620073</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -1259,51 +1259,51 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-04-12 09:08:22 GMT+8</t>
+          <t>2026-04-17 17:27:36 GMT+8</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-04-12 09:09:16 GMT+8</t>
+          <t>2026-04-17 17:37:16 GMT+8</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>2026-04-12 09:06:03 GMT+8</t>
+          <t>2026-04-17 17:26:41 GMT+8</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>2026-04-12 09:06:03 GMT+8</t>
+          <t>2026-04-17 17:26:40 GMT+8</t>
         </is>
       </c>
       <c r="M8" t="n">
-        <v>33014</v>
+        <v>36741</v>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>2026-04-12 09:09:16 GMT+8</t>
+          <t>2026-04-17 17:27:36 GMT+8</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>Hari ini, saya memilih untuk menyebarkan kebaikan dengan membantu jiran mengangkat barang dan berkongsi rezeki dengan rakan. Walaupun kecil, saya percaya setiap kebaikan mampu memberi makna kepada orang lain.</t>
+          <t>Saya menolong pesakit setiap hari</t>
         </is>
       </c>
       <c r="P8" t="n">
-        <v>208</v>
+        <v>33</v>
       </c>
       <c r="Q8" t="n">
-        <v>10.2</v>
+        <v>10.82</v>
       </c>
       <c r="R8" t="n">
-        <v>5.2</v>
+        <v>0.825</v>
       </c>
       <c r="S8" t="n">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="T8" t="n">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="U8" t="n">
         <v>0</v>
@@ -1312,16 +1312,16 @@
         <v>0</v>
       </c>
       <c r="W8" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="X8" t="n">
         <v>0</v>
       </c>
       <c r="Y8" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="Z8" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AA8" t="n">
         <v>0</v>
@@ -1330,7 +1330,7 @@
         <v>0</v>
       </c>
       <c r="AC8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AD8" t="inlineStr">
         <is>
@@ -1341,12 +1341,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Lee Pei Ting</t>
+          <t>Suhaida M Sobri</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>25465212196488673</t>
+          <t>26458022533837392</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -1369,51 +1369,51 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-04-11 10:00:06 GMT+8</t>
+          <t>2026-04-12 08:53:26 GMT+8</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-04-11 10:00:36 GMT+8</t>
+          <t>2026-04-12 09:12:09 GMT+8</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>2026-04-11 09:59:11 GMT+8</t>
+          <t>2026-04-12 09:11:11 GMT+8</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>2026-04-11 09:59:11 GMT+8</t>
+          <t>2026-04-12 08:52:39 GMT+8</t>
         </is>
       </c>
       <c r="M9" t="n">
-        <v>32591</v>
+        <v>33027</v>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>2026-04-11 10:00:06 GMT+8</t>
+          <t>2026-04-12 09:12:09 GMT+8</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>Say suka bersukan dengan keluarga dan kawan kawan.</t>
+          <t>Saya membantu ibuprofen bapa</t>
         </is>
       </c>
       <c r="P9" t="n">
-        <v>50</v>
+        <v>28</v>
       </c>
       <c r="Q9" t="n">
-        <v>11.25</v>
+        <v>15.7</v>
       </c>
       <c r="R9" t="n">
-        <v>1.25</v>
+        <v>0.7000000000000001</v>
       </c>
       <c r="S9" t="n">
         <v>10</v>
       </c>
       <c r="T9" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="U9" t="n">
         <v>0</v>
@@ -1431,7 +1431,7 @@
         <v>2</v>
       </c>
       <c r="Z9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA9" t="n">
         <v>0</v>
@@ -1451,12 +1451,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Lukman Haqem</t>
+          <t>Syikin Supian</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>26297421923276894</t>
+          <t>26634227206261458</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -1479,45 +1479,45 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-03-15 21:32:54 GMT+8</t>
+          <t>2026-04-17 14:53:14 GMT+8</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-03-15 21:33:49 GMT+8</t>
+          <t>2026-04-17 14:53:54 GMT+8</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>2026-03-15 21:32:09 GMT+8</t>
+          <t>2026-04-17 14:50:13 GMT+8</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>2026-03-15 21:31:38 GMT+8</t>
+          <t>2026-04-17 14:49:30 GMT+8</t>
         </is>
       </c>
       <c r="M10" t="n">
-        <v>14126</v>
+        <v>36377</v>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>2026-03-15 21:32:54 GMT+8</t>
+          <t>2026-04-17 14:53:54 GMT+8</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>Saya cuti untuk family</t>
+          <t>Saya suka bawa keluarga menjelajah ke luar negara &amp; ke tempat baru bagi mengenal dunia luar dan pengalaman yang hebat</t>
         </is>
       </c>
       <c r="P10" t="n">
-        <v>22</v>
+        <v>117</v>
       </c>
       <c r="Q10" t="n">
-        <v>10.55</v>
+        <v>-8.07</v>
       </c>
       <c r="R10" t="n">
-        <v>0.55</v>
+        <v>2.925</v>
       </c>
       <c r="S10" t="n">
         <v>10</v>
@@ -1529,10 +1529,10 @@
         <v>0</v>
       </c>
       <c r="V10" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="W10" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="X10" t="n">
         <v>0</v>
@@ -1547,10 +1547,10 @@
         <v>0</v>
       </c>
       <c r="AB10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AC10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AD10" t="inlineStr">
         <is>
@@ -1561,12 +1561,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Maria Muhayadin</t>
+          <t>Sylvia Hsuanfu Chen</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>26575694985402794</t>
+          <t>26550612654593061</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -1589,51 +1589,51 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-04-11 10:02:23 GMT+8</t>
+          <t>2026-04-11 09:03:27 GMT+8</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-04-11 10:02:58 GMT+8</t>
+          <t>2026-04-11 09:04:04 GMT+8</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>2026-04-11 10:01:46 GMT+8</t>
+          <t>2026-04-11 09:02:47 GMT+8</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>2026-04-11 10:01:46 GMT+8</t>
+          <t>2026-04-11 09:00:42 GMT+8</t>
         </is>
       </c>
       <c r="M11" t="n">
-        <v>32596</v>
+        <v>32477</v>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>2026-04-11 10:02:58 GMT+8</t>
+          <t>2026-04-11 09:04:04 GMT+8</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>Saya sangat suka travel bersama keluarga</t>
+          <t>Saya membantu kawan mengangkat barang</t>
         </is>
       </c>
       <c r="P11" t="n">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="Q11" t="n">
-        <v>11</v>
+        <v>15.92</v>
       </c>
       <c r="R11" t="n">
-        <v>1</v>
+        <v>0.925</v>
       </c>
       <c r="S11" t="n">
         <v>10</v>
       </c>
       <c r="T11" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="U11" t="n">
         <v>0</v>
@@ -1651,7 +1651,7 @@
         <v>2</v>
       </c>
       <c r="Z11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA11" t="n">
         <v>0</v>
@@ -1671,12 +1671,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Mar Zu</t>
+          <t>Syuhaida Ahmad</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>26542654198703925</t>
+          <t>26859903310314159</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -1699,51 +1699,51 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>2026-03-30 22:22:02 GMT+8</t>
+          <t>2026-04-17 15:49:59 GMT+8</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-03-30 22:22:42 GMT+8</t>
+          <t>2026-04-17 15:50:27 GMT+8</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>2026-03-30 22:21:26 GMT+8</t>
+          <t>2026-04-17 15:49:20 GMT+8</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>2026-03-30 22:21:25 GMT+8</t>
+          <t>2026-04-17 15:49:20 GMT+8</t>
         </is>
       </c>
       <c r="M12" t="n">
-        <v>26429</v>
+        <v>36524</v>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>2026-03-30 22:22:02 GMT+8</t>
+          <t>2026-04-17 15:50:27 GMT+8</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>Saya membantu kawan mengemas Rumah</t>
+          <t>saya suka travel bersama keluarga</t>
         </is>
       </c>
       <c r="P12" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="Q12" t="n">
-        <v>15.85</v>
+        <v>-14.18</v>
       </c>
       <c r="R12" t="n">
-        <v>0.85</v>
+        <v>0.825</v>
       </c>
       <c r="S12" t="n">
         <v>10</v>
       </c>
       <c r="T12" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="U12" t="n">
         <v>0</v>
@@ -1752,7 +1752,7 @@
         <v>0</v>
       </c>
       <c r="W12" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="X12" t="n">
         <v>0</v>
@@ -1761,7 +1761,7 @@
         <v>2</v>
       </c>
       <c r="Z12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA12" t="n">
         <v>0</v>
@@ -1770,7 +1770,7 @@
         <v>0</v>
       </c>
       <c r="AC12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AD12" t="inlineStr">
         <is>
@@ -1781,12 +1781,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Md</t>
+          <t>TiRa TyRapis</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>26364307709820114</t>
+          <t>26781159228212550</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -1809,52 +1809,52 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2026-02-18 17:19:14 GMT+8</t>
+          <t>2026-04-17 15:06:43 GMT+8</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-02-18 17:21:03 GMT+8</t>
+          <t>2026-04-17 16:40:59 GMT+8</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>2026-02-19 17:18:14 GMT+8</t>
+          <t>2026-04-17 15:05:43 GMT+8</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>2026-02-18 17:16:43 GMT+8</t>
+          <t>2026-04-17 15:05:42 GMT+8</t>
         </is>
       </c>
       <c r="M13" t="n">
-        <v>122</v>
+        <v>36412</v>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>2026-02-18 17:19:14 GMT+8</t>
+          <t>2026-04-17 15:06:43 GMT+8</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>Menolong anak saudara membersih dan menghias rumah untuk hari persandingannya nanti Dan berkongsi Tropicana Twister bersama mereka.</t>
+          <t>saya bantu jiran angkat barang</t>
         </is>
       </c>
       <c r="P13" t="n">
-        <v>131</v>
+        <v>30</v>
       </c>
       <c r="Q13" t="n">
-        <v>18.27</v>
+        <v>-9.25</v>
       </c>
       <c r="R13" t="n">
-        <v>3.275</v>
+        <v>0.75</v>
       </c>
       <c r="S13" t="n">
+        <v>10</v>
+      </c>
+      <c r="T13" t="n">
         <v>5</v>
       </c>
-      <c r="T13" t="n">
-        <v>10</v>
-      </c>
       <c r="U13" t="n">
         <v>0</v>
       </c>
@@ -1862,16 +1862,16 @@
         <v>0</v>
       </c>
       <c r="W13" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="X13" t="n">
         <v>0</v>
       </c>
       <c r="Y13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Z13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AA13" t="n">
         <v>0</v>
@@ -1880,7 +1880,7 @@
         <v>0</v>
       </c>
       <c r="AC13" t="n">
-        <v>1</v>
+        <v>37</v>
       </c>
       <c r="AD13" t="inlineStr">
         <is>
@@ -1891,12 +1891,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Mohamad</t>
+          <t>Wan</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>25200891936250786</t>
+          <t>25907261565595353</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -1919,51 +1919,51 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>2026-02-18 14:32:20 GMT+8</t>
+          <t>2026-02-22 14:50:21 GMT+8</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-02-18 14:33:31 GMT+8</t>
+          <t>2026-02-22 14:51:35 GMT+8</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>2026-02-18 14:30:40 GMT+8</t>
+          <t>2026-02-22 14:48:07 GMT+8</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>2026-02-18 14:29:35 GMT+8</t>
+          <t>2026-02-22 14:48:07 GMT+8</t>
         </is>
       </c>
       <c r="M14" t="n">
-        <v>114</v>
+        <v>460</v>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>2026-02-18 14:32:20 GMT+8</t>
+          <t>2026-02-22 14:50:21 GMT+8</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>saya belanja mak saya sarapan di kedai makan arini</t>
+          <t>Saya bantu isteri saya dengan menyediakan persiapan berbuka dengan Tropicana Twister</t>
         </is>
       </c>
       <c r="P14" t="n">
-        <v>50</v>
+        <v>84</v>
       </c>
       <c r="Q14" t="n">
-        <v>11.25</v>
+        <v>-2.9</v>
       </c>
       <c r="R14" t="n">
-        <v>1.25</v>
+        <v>2.1</v>
       </c>
       <c r="S14" t="n">
         <v>10</v>
       </c>
       <c r="T14" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="U14" t="n">
         <v>0</v>
@@ -1975,13 +1975,13 @@
         <v>0</v>
       </c>
       <c r="X14" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="Y14" t="n">
         <v>2</v>
       </c>
       <c r="Z14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA14" t="n">
         <v>0</v>
@@ -2001,12 +2001,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Mohd Hussairi</t>
+          <t>Yana Shyai</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>1154988495</t>
+          <t>2052286716</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -2029,54 +2029,54 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>2026-04-19 13:09:11 GMT+8</t>
+          <t>2026-04-12 07:42:50 GMT+8</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-04-19 13:09:57 GMT+8</t>
+          <t>2026-04-12 07:43:51 GMT+8</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>2026-04-19 13:08:20 GMT+8</t>
+          <t>2026-04-12 07:41:22 GMT+8</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>2026-03-01 07:47:22 GMT+8</t>
+          <t>2026-04-12 07:41:22 GMT+8</t>
         </is>
       </c>
       <c r="M15" t="n">
-        <v>36904</v>
+        <v>32801</v>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>2026-04-19 13:09:11 GMT+8</t>
+          <t>2026-04-12 07:43:51 GMT+8</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>Setiap hari mereka datang, seolah-olah menjadi sebahagian daripada rutin hidup saya. Dari situ saya belajar tentang kasih sayang, tanggungjawab dan rasa syukur. Memberi makan kucing mungkin nampak perkara kecil, tetapi ia mengajar bahawa kebahagiaan kadang-kadang hadir melalui perbuatan yang sederhana.</t>
+          <t>Saya ajak kawan joging bersama</t>
         </is>
       </c>
       <c r="P15" t="n">
-        <v>303</v>
+        <v>30</v>
       </c>
       <c r="Q15" t="n">
-        <v>26.58</v>
+        <v>10.75</v>
       </c>
       <c r="R15" t="n">
-        <v>7.575</v>
+        <v>0.75</v>
       </c>
       <c r="S15" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="T15" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="U15" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="V15" t="n">
         <v>0</v>
@@ -2088,13 +2088,13 @@
         <v>0</v>
       </c>
       <c r="Y15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Z15" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AA15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB15" t="n">
         <v>0</v>
@@ -2111,12 +2111,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Mohd Khairul Hafiz</t>
+          <t>Yew Teik Ooi</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>26655419207422712</t>
+          <t>25959187133748235</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -2139,48 +2139,48 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>2026-04-12 08:35:12 GMT+8</t>
+          <t>2026-03-29 08:58:47 GMT+8</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-04-12 08:36:46 GMT+8</t>
+          <t>2026-03-29 08:59:53 GMT+8</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>2026-04-12 08:33:41 GMT+8</t>
+          <t>2026-03-29 08:56:27 GMT+8</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>2026-04-12 08:33:41 GMT+8</t>
+          <t>2026-03-08 13:23:13 GMT+8</t>
         </is>
       </c>
       <c r="M16" t="n">
-        <v>32901</v>
+        <v>25339</v>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>2026-04-12 08:35:12 GMT+8</t>
+          <t>2026-03-29 08:59:53 GMT+8</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>Saya suka tropicana sebab air perisa oren dia mempunyai vitamin C dan sesuai untuk seisi keluarga</t>
+          <t>https://scontent.xx.fbcdn.net/v/t1.15752-9/655259381_1509397003947702_5715411122766662692_n.jpg?_nc_cat=109&amp;ccb=1-7&amp;_nc_sid=eb2e90&amp;_nc_ohc=nIXPDVMN0CQQ7kNvwEyEs84&amp;_nc_oc=Adpdu15_SeM5seebYZFm0zJqPTIk2pDpLeigTPzRhgK0pMri1HN-EQ9dQFWyoAvpdqD9mexiwiY3t8z2FaDTb0Ib&amp;_nc_ad=z-m&amp;_nc_cid=0&amp;_nc_zt=23&amp;_nc_ht=scontent.xx&amp;_nc_ss=7a30f&amp;oh=03_Q7cD4wG0wQnb6Q8Fq7oEJl7RKPmiITSDGB1zuNEfz3p0Wdm__A&amp;oe=69F0005F</t>
         </is>
       </c>
       <c r="P16" t="n">
-        <v>97</v>
+        <v>390</v>
       </c>
       <c r="Q16" t="n">
-        <v>-7.57</v>
+        <v>9.75</v>
       </c>
       <c r="R16" t="n">
-        <v>2.425</v>
+        <v>9.75</v>
       </c>
       <c r="S16" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="T16" t="n">
         <v>0</v>
@@ -2195,10 +2195,10 @@
         <v>0</v>
       </c>
       <c r="X16" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="Y16" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Z16" t="n">
         <v>0</v>
@@ -2221,12 +2221,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Muhamad</t>
+          <t>Yna Ahmad</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>26808587638745229</t>
+          <t>27104147162510482</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -2249,52 +2249,52 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>2026-02-20 12:44:58 GMT+8</t>
+          <t>2026-04-12 08:45:02 GMT+8</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-02-20 12:48:00 GMT+8</t>
+          <t>2026-04-12 09:16:15 GMT+8</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>2026-02-20 12:39:36 GMT+8</t>
+          <t>2026-04-12 09:14:27 GMT+8</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>2026-02-20 12:39:36 GMT+8</t>
+          <t>2026-04-12 08:43:22 GMT+8</t>
         </is>
       </c>
       <c r="M17" t="n">
-        <v>226</v>
+        <v>33041</v>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>2026-02-20 12:48:00 GMT+8</t>
+          <t>2026-04-12 09:16:15 GMT+8</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>Sempena bulan puasa, kita boleh memperbanyakkan ibadah, bersedekah kepada yang memerlukan dan meluangkan masa bersama keluarga. Selain itu, kita juga boleh menjaga akhlak serta memperbaiki diri agar Ramadan lebih bermakna. 🌙✨</t>
+          <t>Saling membantu antara satu sama lain dalam kehidupan.</t>
         </is>
       </c>
       <c r="P17" t="n">
-        <v>225</v>
+        <v>54</v>
       </c>
       <c r="Q17" t="n">
-        <v>10.62</v>
+        <v>6.35</v>
       </c>
       <c r="R17" t="n">
-        <v>5.625</v>
+        <v>1.35</v>
       </c>
       <c r="S17" t="n">
+        <v>0</v>
+      </c>
+      <c r="T17" t="n">
         <v>5</v>
       </c>
-      <c r="T17" t="n">
-        <v>0</v>
-      </c>
       <c r="U17" t="n">
         <v>0</v>
       </c>
@@ -2308,10 +2308,10 @@
         <v>0</v>
       </c>
       <c r="Y17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Z17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA17" t="n">
         <v>0</v>
@@ -2331,12 +2331,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Muhammad Zazmie Bin Amirudin</t>
+          <t>Zucc</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>26763040910027742</t>
+          <t>26345565091716286</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -2359,45 +2359,45 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>2026-04-17 15:50:53 GMT+8</t>
+          <t>2026-02-16 21:28:53 GMT+8</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-04-17 16:15:11 GMT+8</t>
+          <t>2026-02-16 21:29:28 GMT+8</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>2026-04-17 15:50:14 GMT+8</t>
+          <t>2026-02-16 21:28:11 GMT+8</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>2026-04-17 15:50:14 GMT+8</t>
+          <t>2026-02-16 21:28:10 GMT+8</t>
         </is>
       </c>
       <c r="M18" t="n">
-        <v>36526</v>
+        <v>61</v>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>2026-04-17 15:50:53 GMT+8</t>
+          <t>2026-02-16 21:28:53 GMT+8</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>saya tolong tukar tayar kereta isteri</t>
+          <t>Saya bantu ibu membersihkan rumah hari ini.</t>
         </is>
       </c>
       <c r="P18" t="n">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="Q18" t="n">
-        <v>15.92</v>
+        <v>16.08</v>
       </c>
       <c r="R18" t="n">
-        <v>0.925</v>
+        <v>1.075</v>
       </c>
       <c r="S18" t="n">
         <v>10</v>
@@ -2441,25 +2441,25 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Muhd Rashid</t>
+          <t>Aji</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>26335725386088254</t>
+          <t>1917989543</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D19" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E19" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F19" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G19" t="n">
         <v>25</v>
@@ -2469,48 +2469,48 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>2026-04-17 14:07:10 GMT+8</t>
+          <t>2026-02-19 17:04:51 GMT+8</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-04-17 14:09:48 GMT+8</t>
+          <t>2026-02-19 17:04:51 GMT+8</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>2026-04-17 14:09:16 GMT+8</t>
+          <t>2026-02-22 22:28:53 GMT+8</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>2026-04-17 14:06:02 GMT+8</t>
+          <t>2026-02-16 14:51:03 GMT+8</t>
         </is>
       </c>
       <c r="M19" t="n">
-        <v>36063</v>
+        <v>183</v>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>2026-04-17 14:07:10 GMT+8</t>
+          <t>2026-02-19 17:04:51 GMT+8</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>Saya suka membantu isteri saya dan keluarga</t>
+          <t>Kongsi nikmat oren Tropicana sewaktu berbuka.</t>
         </is>
       </c>
       <c r="P19" t="n">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="Q19" t="n">
-        <v>21.08</v>
+        <v>-13.88</v>
       </c>
       <c r="R19" t="n">
-        <v>1.075</v>
+        <v>1.125</v>
       </c>
       <c r="S19" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="T19" t="n">
         <v>5</v>
@@ -2525,10 +2525,10 @@
         <v>0</v>
       </c>
       <c r="X19" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="Y19" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="Z19" t="n">
         <v>1</v>
@@ -2551,25 +2551,25 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Must Leyzha</t>
+          <t>Marzuki Sha'ari</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>26109445212060830</t>
+          <t>26810473041893266</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E20" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F20" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G20" t="n">
         <v>25</v>
@@ -2579,51 +2579,51 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>2026-04-12 09:21:24 GMT+8</t>
+          <t>2026-03-06 17:29:08 GMT+8</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-04-12 09:23:26 GMT+8</t>
+          <t>2026-03-06 17:29:08 GMT+8</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>2026-04-12 09:19:10 GMT+8</t>
+          <t>2026-03-06 17:25:00 GMT+8</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>2026-04-12 09:19:10 GMT+8</t>
+          <t>2026-03-06 17:25:00 GMT+8</t>
         </is>
       </c>
       <c r="M20" t="n">
-        <v>33058</v>
+        <v>6191</v>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>2026-04-12 09:21:24 GMT+8</t>
+          <t>2026-03-06 17:29:08 GMT+8</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>Saya kongsikan Tropicana Twister bersama rakan untuk sebarkan keenakan rasa dari setiap tegukan.</t>
+          <t>Saya membantu jiran saya memotong rumput</t>
         </is>
       </c>
       <c r="P20" t="n">
-        <v>96</v>
+        <v>40</v>
       </c>
       <c r="Q20" t="n">
-        <v>-7.6</v>
+        <v>16</v>
       </c>
       <c r="R20" t="n">
-        <v>2.4</v>
+        <v>1</v>
       </c>
       <c r="S20" t="n">
         <v>10</v>
       </c>
       <c r="T20" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="U20" t="n">
         <v>0</v>
@@ -2635,13 +2635,13 @@
         <v>0</v>
       </c>
       <c r="X20" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="Y20" t="n">
         <v>2</v>
       </c>
       <c r="Z20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA20" t="n">
         <v>0</v>
@@ -2661,25 +2661,25 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Najwan Amir</t>
+          <t>Unta Demam</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>26430102329933476</t>
+          <t>27175029105413988</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D21" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E21" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F21" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G21" t="n">
         <v>25</v>
@@ -2689,54 +2689,54 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>2026-04-17 14:18:56 GMT+8</t>
+          <t>2026-04-13 08:06:02 GMT+8</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-04-17 14:19:48 GMT+8</t>
+          <t>2026-04-13 08:06:02 GMT+8</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>2026-04-17 14:18:02 GMT+8</t>
+          <t>2026-04-10 13:19:03 GMT+8</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>2026-04-17 14:18:01 GMT+8</t>
+          <t>2026-04-10 12:50:18 GMT+8</t>
         </is>
       </c>
       <c r="M21" t="n">
-        <v>36181</v>
+        <v>33328</v>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>2026-04-17 14:18:56 GMT+8</t>
+          <t>2026-04-13 08:06:02 GMT+8</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>Saya suka belanja family makan kerana buat mereka gembira</t>
+          <t>Harini saya mendermakan RM1 kepada Masjid Bandar Utama melalui kod qr. Saya harap dapat konsisten setiap hari menderma RM1 kepada mana mana masjid kerana saya bukanlah orang yang berada dan percaya kepada konsisten melakukan kebaikan walau sedikit.</t>
         </is>
       </c>
       <c r="P21" t="n">
-        <v>57</v>
+        <v>248</v>
       </c>
       <c r="Q21" t="n">
-        <v>20.42</v>
+        <v>16.2</v>
       </c>
       <c r="R21" t="n">
-        <v>1.425</v>
+        <v>6.2</v>
       </c>
       <c r="S21" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="T21" t="n">
         <v>5</v>
       </c>
       <c r="U21" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="V21" t="n">
         <v>0</v>
@@ -2748,13 +2748,13 @@
         <v>0</v>
       </c>
       <c r="Y21" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Z21" t="n">
         <v>1</v>
       </c>
       <c r="AA21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB21" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
checked for ineligible winners and updated the winners lists
</commit_message>
<xml_diff>
--- a/outputs/replacement_candidates_next_20_with_journals.xlsx
+++ b/outputs/replacement_candidates_next_20_with_journals.xlsx
@@ -571,12 +571,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Shameel Isfahan</t>
+          <t>Siti Nurhani</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>25409058178770177</t>
+          <t>27099866149620073</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -599,51 +599,51 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-04-12 09:57:57 GMT+8</t>
+          <t>2026-04-17 17:27:36 GMT+8</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-04-12 10:26:46 GMT+8</t>
+          <t>2026-04-17 17:37:16 GMT+8</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2026-04-12 09:56:09 GMT+8</t>
+          <t>2026-04-17 17:26:41 GMT+8</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2026-04-12 09:56:08 GMT+8</t>
+          <t>2026-04-17 17:26:40 GMT+8</t>
         </is>
       </c>
       <c r="M2" t="n">
-        <v>33118</v>
+        <v>36741</v>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-04-12 09:57:57 GMT+8</t>
+          <t>2026-04-17 17:27:36 GMT+8</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>Saya suka berlari sambil bersedekah</t>
+          <t>Saya menolong pesakit setiap hari</t>
         </is>
       </c>
       <c r="P2" t="n">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="Q2" t="n">
-        <v>5.88</v>
+        <v>10.82</v>
       </c>
       <c r="R2" t="n">
-        <v>0.875</v>
+        <v>0.825</v>
       </c>
       <c r="S2" t="n">
         <v>5</v>
       </c>
       <c r="T2" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="U2" t="n">
         <v>0</v>
@@ -661,7 +661,7 @@
         <v>1</v>
       </c>
       <c r="Z2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA2" t="n">
         <v>0</v>
@@ -681,12 +681,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Shazlin Rosly</t>
+          <t>Suhaida M Sobri</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>26809398435345201</t>
+          <t>26458022533837392</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -709,45 +709,45 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-04-12 08:22:19 GMT+8</t>
+          <t>2026-04-12 08:53:26 GMT+8</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-04-12 08:22:53 GMT+8</t>
+          <t>2026-04-12 09:12:09 GMT+8</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>2026-04-12 08:20:50 GMT+8</t>
+          <t>2026-04-12 09:11:11 GMT+8</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>2026-04-12 08:20:49 GMT+8</t>
+          <t>2026-04-12 08:52:39 GMT+8</t>
         </is>
       </c>
       <c r="M3" t="n">
-        <v>32871</v>
+        <v>33027</v>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-04-12 08:22:53 GMT+8</t>
+          <t>2026-04-12 09:12:09 GMT+8</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Saya Bantu jiran angkat air</t>
+          <t>Saya membantu ibuprofen bapa</t>
         </is>
       </c>
       <c r="P3" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="Q3" t="n">
-        <v>15.68</v>
+        <v>15.7</v>
       </c>
       <c r="R3" t="n">
-        <v>0.6749999999999999</v>
+        <v>0.7000000000000001</v>
       </c>
       <c r="S3" t="n">
         <v>10</v>
@@ -791,12 +791,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Shera Nazri</t>
+          <t>Syikin Supian</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>187412901</t>
+          <t>26634227206261458</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -819,60 +819,60 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-03-16 05:58:14 GMT+8</t>
+          <t>2026-04-17 14:53:14 GMT+8</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-03-16 05:58:47 GMT+8</t>
+          <t>2026-04-17 14:53:54 GMT+8</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>2026-04-03 13:41:35 GMT+8</t>
+          <t>2026-04-17 14:50:13 GMT+8</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>2026-03-16 05:56:01 GMT+8</t>
+          <t>2026-04-17 14:49:30 GMT+8</t>
         </is>
       </c>
       <c r="M4" t="n">
-        <v>14177</v>
+        <v>36377</v>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>2026-03-16 05:58:47 GMT+8</t>
+          <t>2026-04-17 14:53:54 GMT+8</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>Saya bantu keluarga saya mengecat rumah</t>
+          <t>Saya suka bawa keluarga menjelajah ke luar negara &amp; ke tempat baru bagi mengenal dunia luar dan pengalaman yang hebat</t>
         </is>
       </c>
       <c r="P4" t="n">
-        <v>39</v>
+        <v>117</v>
       </c>
       <c r="Q4" t="n">
-        <v>15.98</v>
+        <v>-8.07</v>
       </c>
       <c r="R4" t="n">
-        <v>0.9750000000000001</v>
+        <v>2.925</v>
       </c>
       <c r="S4" t="n">
         <v>10</v>
       </c>
       <c r="T4" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="U4" t="n">
         <v>0</v>
       </c>
       <c r="V4" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="W4" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="X4" t="n">
         <v>0</v>
@@ -881,16 +881,16 @@
         <v>2</v>
       </c>
       <c r="Z4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA4" t="n">
         <v>0</v>
       </c>
       <c r="AB4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AC4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AD4" t="inlineStr">
         <is>
@@ -901,12 +901,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Shira Jalil</t>
+          <t>Sylvia Hsuanfu Chen</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>26304478562497060</t>
+          <t>26550612654593061</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -929,48 +929,48 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-03-14 01:22:42 GMT+8</t>
+          <t>2026-04-11 09:03:27 GMT+8</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-03-14 01:24:53 GMT+8</t>
+          <t>2026-04-11 09:04:04 GMT+8</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>2026-03-14 01:24:08 GMT+8</t>
+          <t>2026-04-11 09:02:47 GMT+8</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>2026-03-14 01:21:38 GMT+8</t>
+          <t>2026-04-11 09:00:42 GMT+8</t>
         </is>
       </c>
       <c r="M5" t="n">
-        <v>11836</v>
+        <v>32477</v>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>2026-03-14 01:24:53 GMT+8</t>
+          <t>2026-04-11 09:04:04 GMT+8</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>saya suka tolong orang</t>
+          <t>Saya membantu kawan mengangkat barang</t>
         </is>
       </c>
       <c r="P5" t="n">
-        <v>22</v>
+        <v>37</v>
       </c>
       <c r="Q5" t="n">
-        <v>-14.45</v>
+        <v>15.92</v>
       </c>
       <c r="R5" t="n">
-        <v>0.55</v>
+        <v>0.925</v>
       </c>
       <c r="S5" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="T5" t="n">
         <v>5</v>
@@ -982,13 +982,13 @@
         <v>0</v>
       </c>
       <c r="W5" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="X5" t="n">
         <v>0</v>
       </c>
       <c r="Y5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Z5" t="n">
         <v>1</v>
@@ -1000,7 +1000,7 @@
         <v>0</v>
       </c>
       <c r="AC5" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="AD5" t="inlineStr">
         <is>
@@ -1011,12 +1011,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Siew</t>
+          <t>Syuhaida Ahmad</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>765882994</t>
+          <t>26859903310314159</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -1039,48 +1039,48 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-02-20 12:39:13 GMT+8</t>
+          <t>2026-04-17 15:49:59 GMT+8</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-02-20 12:41:25 GMT+8</t>
+          <t>2026-04-17 15:50:27 GMT+8</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>2026-02-20 12:34:32 GMT+8</t>
+          <t>2026-04-17 15:49:20 GMT+8</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>2026-02-20 12:33:49 GMT+8</t>
+          <t>2026-04-17 15:49:20 GMT+8</t>
         </is>
       </c>
       <c r="M6" t="n">
-        <v>220</v>
+        <v>36524</v>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>2026-02-20 12:39:13 GMT+8</t>
+          <t>2026-04-17 15:50:27 GMT+8</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>Saya memperkenalkan minuman tropicana Twister kepada kawan sekerja saya. Selain itu, Tropicana Twister merupakan minuman utama tajaan saya kepada jamuan di anak sekolah saya.</t>
+          <t>saya suka travel bersama keluarga</t>
         </is>
       </c>
       <c r="P6" t="n">
-        <v>174</v>
+        <v>33</v>
       </c>
       <c r="Q6" t="n">
-        <v>19.35</v>
+        <v>-14.18</v>
       </c>
       <c r="R6" t="n">
-        <v>4.35</v>
+        <v>0.825</v>
       </c>
       <c r="S6" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="T6" t="n">
         <v>0</v>
@@ -1092,13 +1092,13 @@
         <v>0</v>
       </c>
       <c r="W6" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="X6" t="n">
         <v>0</v>
       </c>
       <c r="Y6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Z6" t="n">
         <v>0</v>
@@ -1110,7 +1110,7 @@
         <v>0</v>
       </c>
       <c r="AC6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AD6" t="inlineStr">
         <is>
@@ -1121,12 +1121,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Siti Nurhani</t>
+          <t>TiRa TyRapis</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>27099866149620073</t>
+          <t>26781159228212550</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -1149,48 +1149,48 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-04-17 17:27:36 GMT+8</t>
+          <t>2026-04-17 15:06:43 GMT+8</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-04-17 17:37:16 GMT+8</t>
+          <t>2026-04-17 16:40:59 GMT+8</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>2026-04-17 17:26:41 GMT+8</t>
+          <t>2026-04-17 15:05:43 GMT+8</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>2026-04-17 17:26:40 GMT+8</t>
+          <t>2026-04-17 15:05:42 GMT+8</t>
         </is>
       </c>
       <c r="M7" t="n">
-        <v>36741</v>
+        <v>36412</v>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>2026-04-17 17:27:36 GMT+8</t>
+          <t>2026-04-17 15:06:43 GMT+8</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>Saya menolong pesakit setiap hari</t>
+          <t>saya bantu jiran angkat barang</t>
         </is>
       </c>
       <c r="P7" t="n">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="Q7" t="n">
-        <v>10.82</v>
+        <v>-9.25</v>
       </c>
       <c r="R7" t="n">
-        <v>0.825</v>
+        <v>0.75</v>
       </c>
       <c r="S7" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="T7" t="n">
         <v>5</v>
@@ -1202,13 +1202,13 @@
         <v>0</v>
       </c>
       <c r="W7" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="X7" t="n">
         <v>0</v>
       </c>
       <c r="Y7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Z7" t="n">
         <v>1</v>
@@ -1220,7 +1220,7 @@
         <v>0</v>
       </c>
       <c r="AC7" t="n">
-        <v>1</v>
+        <v>37</v>
       </c>
       <c r="AD7" t="inlineStr">
         <is>
@@ -1231,12 +1231,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Suhaida M Sobri</t>
+          <t>Wan</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>26458022533837392</t>
+          <t>25907261565595353</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -1259,45 +1259,45 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-04-12 08:53:26 GMT+8</t>
+          <t>2026-02-22 14:50:21 GMT+8</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-04-12 09:12:09 GMT+8</t>
+          <t>2026-02-22 14:51:35 GMT+8</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>2026-04-12 09:11:11 GMT+8</t>
+          <t>2026-02-22 14:48:07 GMT+8</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>2026-04-12 08:52:39 GMT+8</t>
+          <t>2026-02-22 14:48:07 GMT+8</t>
         </is>
       </c>
       <c r="M8" t="n">
-        <v>33027</v>
+        <v>460</v>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>2026-04-12 09:12:09 GMT+8</t>
+          <t>2026-02-22 14:50:21 GMT+8</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>Saya membantu ibuprofen bapa</t>
+          <t>Saya bantu isteri saya dengan menyediakan persiapan berbuka dengan Tropicana Twister</t>
         </is>
       </c>
       <c r="P8" t="n">
-        <v>28</v>
+        <v>84</v>
       </c>
       <c r="Q8" t="n">
-        <v>15.7</v>
+        <v>-2.9</v>
       </c>
       <c r="R8" t="n">
-        <v>0.7000000000000001</v>
+        <v>2.1</v>
       </c>
       <c r="S8" t="n">
         <v>10</v>
@@ -1315,7 +1315,7 @@
         <v>0</v>
       </c>
       <c r="X8" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="Y8" t="n">
         <v>2</v>
@@ -1341,12 +1341,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Syikin Supian</t>
+          <t>Yana Shyai</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>26634227206261458</t>
+          <t>2052286716</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -1369,45 +1369,45 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-04-17 14:53:14 GMT+8</t>
+          <t>2026-04-12 07:42:50 GMT+8</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-04-17 14:53:54 GMT+8</t>
+          <t>2026-04-12 07:43:51 GMT+8</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>2026-04-17 14:50:13 GMT+8</t>
+          <t>2026-04-12 07:41:22 GMT+8</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>2026-04-17 14:49:30 GMT+8</t>
+          <t>2026-04-12 07:41:22 GMT+8</t>
         </is>
       </c>
       <c r="M9" t="n">
-        <v>36377</v>
+        <v>32801</v>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>2026-04-17 14:53:54 GMT+8</t>
+          <t>2026-04-12 07:43:51 GMT+8</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>Saya suka bawa keluarga menjelajah ke luar negara &amp; ke tempat baru bagi mengenal dunia luar dan pengalaman yang hebat</t>
+          <t>Saya ajak kawan joging bersama</t>
         </is>
       </c>
       <c r="P9" t="n">
-        <v>117</v>
+        <v>30</v>
       </c>
       <c r="Q9" t="n">
-        <v>-8.07</v>
+        <v>10.75</v>
       </c>
       <c r="R9" t="n">
-        <v>2.925</v>
+        <v>0.75</v>
       </c>
       <c r="S9" t="n">
         <v>10</v>
@@ -1419,10 +1419,10 @@
         <v>0</v>
       </c>
       <c r="V9" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="W9" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="X9" t="n">
         <v>0</v>
@@ -1437,10 +1437,10 @@
         <v>0</v>
       </c>
       <c r="AB9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AC9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AD9" t="inlineStr">
         <is>
@@ -1451,12 +1451,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Sylvia Hsuanfu Chen</t>
+          <t>Yew Teik Ooi</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>26550612654593061</t>
+          <t>25959187133748235</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -1479,51 +1479,51 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-04-11 09:03:27 GMT+8</t>
+          <t>2026-03-29 08:58:47 GMT+8</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-04-11 09:04:04 GMT+8</t>
+          <t>2026-03-29 08:59:53 GMT+8</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>2026-04-11 09:02:47 GMT+8</t>
+          <t>2026-03-29 08:56:27 GMT+8</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>2026-04-11 09:00:42 GMT+8</t>
+          <t>2026-03-08 13:23:13 GMT+8</t>
         </is>
       </c>
       <c r="M10" t="n">
-        <v>32477</v>
+        <v>25339</v>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>2026-04-11 09:04:04 GMT+8</t>
+          <t>2026-03-29 08:59:53 GMT+8</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>Saya membantu kawan mengangkat barang</t>
+          <t>https://scontent.xx.fbcdn.net/v/t1.15752-9/655259381_1509397003947702_5715411122766662692_n.jpg?_nc_cat=109&amp;ccb=1-7&amp;_nc_sid=eb2e90&amp;_nc_ohc=nIXPDVMN0CQQ7kNvwEyEs84&amp;_nc_oc=Adpdu15_SeM5seebYZFm0zJqPTIk2pDpLeigTPzRhgK0pMri1HN-EQ9dQFWyoAvpdqD9mexiwiY3t8z2FaDTb0Ib&amp;_nc_ad=z-m&amp;_nc_cid=0&amp;_nc_zt=23&amp;_nc_ht=scontent.xx&amp;_nc_ss=7a30f&amp;oh=03_Q7cD4wG0wQnb6Q8Fq7oEJl7RKPmiITSDGB1zuNEfz3p0Wdm__A&amp;oe=69F0005F</t>
         </is>
       </c>
       <c r="P10" t="n">
-        <v>37</v>
+        <v>390</v>
       </c>
       <c r="Q10" t="n">
-        <v>15.92</v>
+        <v>9.75</v>
       </c>
       <c r="R10" t="n">
-        <v>0.925</v>
+        <v>9.75</v>
       </c>
       <c r="S10" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="T10" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="U10" t="n">
         <v>0</v>
@@ -1538,10 +1538,10 @@
         <v>0</v>
       </c>
       <c r="Y10" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Z10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA10" t="n">
         <v>0</v>
@@ -1561,12 +1561,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Syuhaida Ahmad</t>
+          <t>Yna Ahmad</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>26859903310314159</t>
+          <t>27104147162510482</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -1589,51 +1589,51 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-04-17 15:49:59 GMT+8</t>
+          <t>2026-04-12 08:45:02 GMT+8</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-04-17 15:50:27 GMT+8</t>
+          <t>2026-04-12 09:16:15 GMT+8</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>2026-04-17 15:49:20 GMT+8</t>
+          <t>2026-04-12 09:14:27 GMT+8</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>2026-04-17 15:49:20 GMT+8</t>
+          <t>2026-04-12 08:43:22 GMT+8</t>
         </is>
       </c>
       <c r="M11" t="n">
-        <v>36524</v>
+        <v>33041</v>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>2026-04-17 15:50:27 GMT+8</t>
+          <t>2026-04-12 09:16:15 GMT+8</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>saya suka travel bersama keluarga</t>
+          <t>Saling membantu antara satu sama lain dalam kehidupan.</t>
         </is>
       </c>
       <c r="P11" t="n">
-        <v>33</v>
+        <v>54</v>
       </c>
       <c r="Q11" t="n">
-        <v>-14.18</v>
+        <v>6.35</v>
       </c>
       <c r="R11" t="n">
-        <v>0.825</v>
+        <v>1.35</v>
       </c>
       <c r="S11" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="T11" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="U11" t="n">
         <v>0</v>
@@ -1642,16 +1642,16 @@
         <v>0</v>
       </c>
       <c r="W11" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="X11" t="n">
         <v>0</v>
       </c>
       <c r="Y11" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Z11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA11" t="n">
         <v>0</v>
@@ -1660,7 +1660,7 @@
         <v>0</v>
       </c>
       <c r="AC11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AD11" t="inlineStr">
         <is>
@@ -1671,12 +1671,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>TiRa TyRapis</t>
+          <t>Zucc</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>26781159228212550</t>
+          <t>26345565091716286</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -1699,45 +1699,45 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>2026-04-17 15:06:43 GMT+8</t>
+          <t>2026-02-16 21:28:53 GMT+8</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-04-17 16:40:59 GMT+8</t>
+          <t>2026-02-16 21:29:28 GMT+8</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>2026-04-17 15:05:43 GMT+8</t>
+          <t>2026-02-16 21:28:11 GMT+8</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>2026-04-17 15:05:42 GMT+8</t>
+          <t>2026-02-16 21:28:10 GMT+8</t>
         </is>
       </c>
       <c r="M12" t="n">
-        <v>36412</v>
+        <v>61</v>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>2026-04-17 15:06:43 GMT+8</t>
+          <t>2026-02-16 21:28:53 GMT+8</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>saya bantu jiran angkat barang</t>
+          <t>Saya bantu ibu membersihkan rumah hari ini.</t>
         </is>
       </c>
       <c r="P12" t="n">
-        <v>30</v>
+        <v>43</v>
       </c>
       <c r="Q12" t="n">
-        <v>-9.25</v>
+        <v>16.08</v>
       </c>
       <c r="R12" t="n">
-        <v>0.75</v>
+        <v>1.075</v>
       </c>
       <c r="S12" t="n">
         <v>10</v>
@@ -1752,7 +1752,7 @@
         <v>0</v>
       </c>
       <c r="W12" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="X12" t="n">
         <v>0</v>
@@ -1770,7 +1770,7 @@
         <v>0</v>
       </c>
       <c r="AC12" t="n">
-        <v>37</v>
+        <v>1</v>
       </c>
       <c r="AD12" t="inlineStr">
         <is>
@@ -1781,25 +1781,25 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Wan</t>
+          <t>Aji</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>25907261565595353</t>
+          <t>1917989543</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E13" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F13" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G13" t="n">
         <v>25</v>
@@ -1809,48 +1809,48 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2026-02-22 14:50:21 GMT+8</t>
+          <t>2026-02-19 17:04:51 GMT+8</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-02-22 14:51:35 GMT+8</t>
+          <t>2026-02-19 17:04:51 GMT+8</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>2026-02-22 14:48:07 GMT+8</t>
+          <t>2026-02-22 22:28:53 GMT+8</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>2026-02-22 14:48:07 GMT+8</t>
+          <t>2026-02-16 14:51:03 GMT+8</t>
         </is>
       </c>
       <c r="M13" t="n">
-        <v>460</v>
+        <v>183</v>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>2026-02-22 14:50:21 GMT+8</t>
+          <t>2026-02-19 17:04:51 GMT+8</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>Saya bantu isteri saya dengan menyediakan persiapan berbuka dengan Tropicana Twister</t>
+          <t>Kongsi nikmat oren Tropicana sewaktu berbuka.</t>
         </is>
       </c>
       <c r="P13" t="n">
-        <v>84</v>
+        <v>45</v>
       </c>
       <c r="Q13" t="n">
-        <v>-2.9</v>
+        <v>-13.88</v>
       </c>
       <c r="R13" t="n">
-        <v>2.1</v>
+        <v>1.125</v>
       </c>
       <c r="S13" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="T13" t="n">
         <v>5</v>
@@ -1868,7 +1868,7 @@
         <v>20</v>
       </c>
       <c r="Y13" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Z13" t="n">
         <v>1</v>
@@ -1891,25 +1891,25 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Yana Shyai</t>
+          <t>Marzuki Sha'ari</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2052286716</t>
+          <t>26810473041893266</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D14" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E14" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F14" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G14" t="n">
         <v>25</v>
@@ -1919,51 +1919,51 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>2026-04-12 07:42:50 GMT+8</t>
+          <t>2026-03-06 17:29:08 GMT+8</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-04-12 07:43:51 GMT+8</t>
+          <t>2026-03-06 17:29:08 GMT+8</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>2026-04-12 07:41:22 GMT+8</t>
+          <t>2026-03-06 17:25:00 GMT+8</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>2026-04-12 07:41:22 GMT+8</t>
+          <t>2026-03-06 17:25:00 GMT+8</t>
         </is>
       </c>
       <c r="M14" t="n">
-        <v>32801</v>
+        <v>6191</v>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>2026-04-12 07:43:51 GMT+8</t>
+          <t>2026-03-06 17:29:08 GMT+8</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>Saya ajak kawan joging bersama</t>
+          <t>Saya membantu jiran saya memotong rumput</t>
         </is>
       </c>
       <c r="P14" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="Q14" t="n">
-        <v>10.75</v>
+        <v>16</v>
       </c>
       <c r="R14" t="n">
-        <v>0.75</v>
+        <v>1</v>
       </c>
       <c r="S14" t="n">
         <v>10</v>
       </c>
       <c r="T14" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="U14" t="n">
         <v>0</v>
@@ -1981,7 +1981,7 @@
         <v>2</v>
       </c>
       <c r="Z14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA14" t="n">
         <v>0</v>
@@ -2001,25 +2001,25 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Yew Teik Ooi</t>
+          <t>Unta Demam</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>25959187133748235</t>
+          <t>27175029105413988</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E15" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F15" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G15" t="n">
         <v>25</v>
@@ -2029,51 +2029,51 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>2026-03-29 08:58:47 GMT+8</t>
+          <t>2026-04-13 08:06:02 GMT+8</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-03-29 08:59:53 GMT+8</t>
+          <t>2026-04-13 08:06:02 GMT+8</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>2026-03-29 08:56:27 GMT+8</t>
+          <t>2026-04-10 13:19:03 GMT+8</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>2026-03-08 13:23:13 GMT+8</t>
+          <t>2026-04-10 12:50:18 GMT+8</t>
         </is>
       </c>
       <c r="M15" t="n">
-        <v>25339</v>
+        <v>33328</v>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>2026-03-29 08:59:53 GMT+8</t>
+          <t>2026-04-13 08:06:02 GMT+8</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>https://scontent.xx.fbcdn.net/v/t1.15752-9/655259381_1509397003947702_5715411122766662692_n.jpg?_nc_cat=109&amp;ccb=1-7&amp;_nc_sid=eb2e90&amp;_nc_ohc=nIXPDVMN0CQQ7kNvwEyEs84&amp;_nc_oc=Adpdu15_SeM5seebYZFm0zJqPTIk2pDpLeigTPzRhgK0pMri1HN-EQ9dQFWyoAvpdqD9mexiwiY3t8z2FaDTb0Ib&amp;_nc_ad=z-m&amp;_nc_cid=0&amp;_nc_zt=23&amp;_nc_ht=scontent.xx&amp;_nc_ss=7a30f&amp;oh=03_Q7cD4wG0wQnb6Q8Fq7oEJl7RKPmiITSDGB1zuNEfz3p0Wdm__A&amp;oe=69F0005F</t>
+          <t>Harini saya mendermakan RM1 kepada Masjid Bandar Utama melalui kod qr. Saya harap dapat konsisten setiap hari menderma RM1 kepada mana mana masjid kerana saya bukanlah orang yang berada dan percaya kepada konsisten melakukan kebaikan walau sedikit.</t>
         </is>
       </c>
       <c r="P15" t="n">
-        <v>390</v>
+        <v>248</v>
       </c>
       <c r="Q15" t="n">
-        <v>9.75</v>
+        <v>16.2</v>
       </c>
       <c r="R15" t="n">
-        <v>9.75</v>
+        <v>6.2</v>
       </c>
       <c r="S15" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="T15" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="U15" t="n">
         <v>0</v>
@@ -2088,10 +2088,10 @@
         <v>0</v>
       </c>
       <c r="Y15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA15" t="n">
         <v>0</v>
@@ -2111,79 +2111,79 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Yna Ahmad</t>
+          <t>Aini</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>27104147162510482</t>
+          <t>26602935525965782</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G16" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="H16" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>2026-04-12 08:45:02 GMT+8</t>
+          <t>2026-04-04 23:04:41 GMT+8</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-04-12 09:16:15 GMT+8</t>
+          <t>2026-04-04 23:04:41 GMT+8</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>2026-04-12 09:14:27 GMT+8</t>
+          <t>2026-02-17 20:20:35 GMT+8</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>2026-04-12 08:43:22 GMT+8</t>
+          <t>2026-02-17 20:18:18 GMT+8</t>
         </is>
       </c>
       <c r="M16" t="n">
-        <v>33041</v>
+        <v>30083</v>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>2026-04-12 09:16:15 GMT+8</t>
+          <t>2026-04-04 23:04:41 GMT+8</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>Saling membantu antara satu sama lain dalam kehidupan.</t>
+          <t>Saya bersama jiran bergotong-royong memasak untuk rumah terbuka kawasan perumahan kami</t>
         </is>
       </c>
       <c r="P16" t="n">
-        <v>54</v>
+        <v>86</v>
       </c>
       <c r="Q16" t="n">
-        <v>6.35</v>
+        <v>17.15</v>
       </c>
       <c r="R16" t="n">
-        <v>1.35</v>
+        <v>2.15</v>
       </c>
       <c r="S16" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="T16" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="U16" t="n">
         <v>0</v>
@@ -2198,10 +2198,10 @@
         <v>0</v>
       </c>
       <c r="Y16" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="Z16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA16" t="n">
         <v>0</v>
@@ -2221,79 +2221,79 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Zucc</t>
+          <t>Ann Hadid</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>26345565091716286</t>
+          <t>26064885319846636</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G17" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="H17" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>2026-02-16 21:28:53 GMT+8</t>
+          <t>2026-03-06 02:52:06 GMT+8</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-02-16 21:29:28 GMT+8</t>
+          <t>2026-03-06 02:52:06 GMT+8</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>2026-02-16 21:28:11 GMT+8</t>
+          <t>2026-03-04 14:06:55 GMT+8</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>2026-02-16 21:28:10 GMT+8</t>
+          <t>2026-03-04 14:05:40 GMT+8</t>
         </is>
       </c>
       <c r="M17" t="n">
-        <v>61</v>
+        <v>5916</v>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>2026-02-16 21:28:53 GMT+8</t>
+          <t>2026-03-06 02:52:06 GMT+8</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>Saya bantu ibu membersihkan rumah hari ini.</t>
+          <t>Saya selamatkan anak kucing yang terjatuh di dalam longkang,mandikannya &amp; membela nya kerana dia masih kecil dan ibunya tiada.</t>
         </is>
       </c>
       <c r="P17" t="n">
-        <v>43</v>
+        <v>126</v>
       </c>
       <c r="Q17" t="n">
-        <v>16.08</v>
+        <v>13.15</v>
       </c>
       <c r="R17" t="n">
-        <v>1.075</v>
+        <v>3.15</v>
       </c>
       <c r="S17" t="n">
         <v>10</v>
       </c>
       <c r="T17" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="U17" t="n">
         <v>0</v>
@@ -2311,7 +2311,7 @@
         <v>2</v>
       </c>
       <c r="Z17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA17" t="n">
         <v>0</v>
@@ -2331,12 +2331,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Aji</t>
+          <t>Fazliana Azman</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>1917989543</t>
+          <t>27489929837273577</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -2346,58 +2346,58 @@
         <v>1</v>
       </c>
       <c r="E18" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F18" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G18" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="H18" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>2026-02-19 17:04:51 GMT+8</t>
+          <t>2026-04-07 22:26:14 GMT+8</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-02-19 17:04:51 GMT+8</t>
+          <t>2026-04-07 22:26:14 GMT+8</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>2026-02-22 22:28:53 GMT+8</t>
+          <t>2026-04-07 22:23:08 GMT+8</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>2026-02-16 14:51:03 GMT+8</t>
+          <t>2026-04-07 13:55:37 GMT+8</t>
         </is>
       </c>
       <c r="M18" t="n">
-        <v>183</v>
+        <v>31353</v>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>2026-02-19 17:04:51 GMT+8</t>
+          <t>2026-04-07 22:26:14 GMT+8</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>Kongsi nikmat oren Tropicana sewaktu berbuka.</t>
+          <t>Dimana mahu kongsi jurnal?</t>
         </is>
       </c>
       <c r="P18" t="n">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="Q18" t="n">
-        <v>-13.88</v>
+        <v>5.65</v>
       </c>
       <c r="R18" t="n">
-        <v>1.125</v>
+        <v>0.65</v>
       </c>
       <c r="S18" t="n">
         <v>0</v>
@@ -2415,7 +2415,7 @@
         <v>0</v>
       </c>
       <c r="X18" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="Y18" t="n">
         <v>0</v>
@@ -2441,12 +2441,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Marzuki Sha'ari</t>
+          <t>Hong Tian</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>26810473041893266</t>
+          <t>26175248618835934</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -2456,64 +2456,64 @@
         <v>1</v>
       </c>
       <c r="E19" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F19" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G19" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="H19" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>2026-03-06 17:29:08 GMT+8</t>
+          <t>2026-03-26 20:51:41 GMT+8</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-03-06 17:29:08 GMT+8</t>
+          <t>2026-03-26 20:51:41 GMT+8</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>2026-03-06 17:25:00 GMT+8</t>
+          <t>2026-03-13 19:22:31 GMT+8</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>2026-03-06 17:25:00 GMT+8</t>
+          <t>2026-03-13 19:22:30 GMT+8</t>
         </is>
       </c>
       <c r="M19" t="n">
-        <v>6191</v>
+        <v>22278</v>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>2026-03-06 17:29:08 GMT+8</t>
+          <t>2026-03-26 20:51:41 GMT+8</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>Saya membantu jiran saya memotong rumput</t>
+          <t>“Saya menderma darah dan menggalak kawan-kawan saya juga menyertai kempen derma darah”</t>
         </is>
       </c>
       <c r="P19" t="n">
-        <v>40</v>
+        <v>86</v>
       </c>
       <c r="Q19" t="n">
-        <v>16</v>
+        <v>7.15</v>
       </c>
       <c r="R19" t="n">
-        <v>1</v>
+        <v>2.15</v>
       </c>
       <c r="S19" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="T19" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="U19" t="n">
         <v>0</v>
@@ -2528,10 +2528,10 @@
         <v>0</v>
       </c>
       <c r="Y19" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Z19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA19" t="n">
         <v>0</v>
@@ -2551,12 +2551,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Unta Demam</t>
+          <t>Izzat Lasim</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>27175029105413988</t>
+          <t>1368751717</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -2566,64 +2566,64 @@
         <v>1</v>
       </c>
       <c r="E20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G20" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="H20" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>2026-04-13 08:06:02 GMT+8</t>
+          <t>2026-04-12 05:46:05 GMT+8</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-04-13 08:06:02 GMT+8</t>
+          <t>2026-04-12 05:46:05 GMT+8</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>2026-04-10 13:19:03 GMT+8</t>
+          <t>2026-04-12 05:45:10 GMT+8</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>2026-04-10 12:50:18 GMT+8</t>
+          <t>2026-02-20 10:50:27 GMT+8</t>
         </is>
       </c>
       <c r="M20" t="n">
-        <v>33328</v>
+        <v>32730</v>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>2026-04-13 08:06:02 GMT+8</t>
+          <t>2026-04-12 05:46:05 GMT+8</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>Harini saya mendermakan RM1 kepada Masjid Bandar Utama melalui kod qr. Saya harap dapat konsisten setiap hari menderma RM1 kepada mana mana masjid kerana saya bukanlah orang yang berada dan percaya kepada konsisten melakukan kebaikan walau sedikit.</t>
+          <t>Mari berpuasa 6syawal.</t>
         </is>
       </c>
       <c r="P20" t="n">
-        <v>248</v>
+        <v>22</v>
       </c>
       <c r="Q20" t="n">
-        <v>16.2</v>
+        <v>0.55</v>
       </c>
       <c r="R20" t="n">
-        <v>6.2</v>
+        <v>0.55</v>
       </c>
       <c r="S20" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="T20" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="U20" t="n">
         <v>0</v>
@@ -2638,10 +2638,10 @@
         <v>0</v>
       </c>
       <c r="Y20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Z20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA20" t="n">
         <v>0</v>
@@ -2661,12 +2661,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Aini</t>
+          <t>Joanne Chay</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>26602935525965782</t>
+          <t>26117305194548131</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -2689,57 +2689,57 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>2026-04-04 23:04:41 GMT+8</t>
+          <t>2026-03-03 14:59:30 GMT+8</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-04-04 23:04:41 GMT+8</t>
+          <t>2026-03-03 14:59:30 GMT+8</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>2026-02-17 20:20:35 GMT+8</t>
+          <t>2026-03-02 13:15:55 GMT+8</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>2026-02-17 20:18:18 GMT+8</t>
+          <t>2026-03-02 13:15:54 GMT+8</t>
         </is>
       </c>
       <c r="M21" t="n">
-        <v>30083</v>
+        <v>4981</v>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>2026-04-04 23:04:41 GMT+8</t>
+          <t>2026-03-03 14:59:30 GMT+8</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>Saya bersama jiran bergotong-royong memasak untuk rumah terbuka kawasan perumahan kami</t>
+          <t>When a 80-pax corporate lunch ended, it wasn’t the finish, it was the start of a Food Rescue Mission. We diverted 42.3 kg of premium surplus food from landfills to those in need. From BBQ Beef and Ikan Goreng Sambal to fruits, grains, and bakery items, every dish became a blessing. This saved 72 kg CO₂e, 63,500 litres of water, and 2.5 kg of scraps went to compost/animal feed. Meals reached Chin Christian Fellowship, City Revival Church Home, and PPR Lembah Subang 1, feeding refugees, orphans, and families. Every gram rescued honors God’s creation and spreads hope. 🌿🌏✨</t>
         </is>
       </c>
       <c r="P21" t="n">
-        <v>86</v>
+        <v>575</v>
       </c>
       <c r="Q21" t="n">
-        <v>17.15</v>
+        <v>27.38</v>
       </c>
       <c r="R21" t="n">
-        <v>2.15</v>
+        <v>14.375</v>
       </c>
       <c r="S21" t="n">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="T21" t="n">
         <v>0</v>
       </c>
       <c r="U21" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="V21" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="W21" t="n">
         <v>0</v>
@@ -2748,16 +2748,16 @@
         <v>0</v>
       </c>
       <c r="Y21" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="Z21" t="n">
         <v>0</v>
       </c>
       <c r="AA21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AC21" t="n">
         <v>1</v>

</xml_diff>